<commit_message>
chore(weekly-sync): auto-pull through 2026-07-26
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Nexlev/business_report_week30.xlsx
+++ b/data/ams_weekly_data/Nexlev/business_report_week30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W92"/>
+  <dimension ref="A1:W93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7904,6 +7904,87 @@
         <v>0</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>FBA80111</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>MR-01_Part</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>B0GYSS16FJ</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>B0GYSS16FJ</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MR-01_Part</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>3</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="n">
+        <v>0</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0</v>
+      </c>
+      <c r="R93" t="n">
+        <v>0</v>
+      </c>
+      <c r="S93" t="n">
+        <v>0</v>
+      </c>
+      <c r="T93" t="n">
+        <v>0</v>
+      </c>
+      <c r="U93" t="n">
+        <v>0</v>
+      </c>
+      <c r="V93" t="n">
+        <v>0</v>
+      </c>
+      <c r="W93" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>